<commit_message>
Enhance build process by adding functions.cpp, updating build command, and modifying initialization logic for new deal generation
</commit_message>
<xml_diff>
--- a/Solitaire Database Definitions.xlsx
+++ b/Solitaire Database Definitions.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49E5838881D62E8C/C Projects/Solitaire/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\C Projects\Solitaire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{FF47FFEE-7710-4C9E-9521-F903133D77B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EDE2296-0E17-444C-854A-D9A2AC42A7CA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6B1D71-007E-43E8-A0ED-2B48C21D7017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{98FEF319-7F55-4DB7-B5AE-0D8519D8C0E1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{98FEF319-7F55-4DB7-B5AE-0D8519D8C0E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Deal_Head" sheetId="1" r:id="rId1"/>
     <sheet name="Deal_Data" sheetId="2" r:id="rId2"/>
     <sheet name="inQ" sheetId="3" r:id="rId3"/>
+    <sheet name="card_0" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>This table contains the original deal of a game.</t>
   </si>
@@ -146,6 +147,42 @@
   </si>
   <si>
     <t>Stop date/time. An entry here indicated that this hand has been completed.</t>
+  </si>
+  <si>
+    <t>card_0</t>
+  </si>
+  <si>
+    <t>This lists the properties of the cards, such as Ace pile order, play prder in tableau. This contains the 'rules' of play</t>
+  </si>
+  <si>
+    <t>cardID</t>
+  </si>
+  <si>
+    <t>face</t>
+  </si>
+  <si>
+    <t>suit</t>
+  </si>
+  <si>
+    <t>nextAce</t>
+  </si>
+  <si>
+    <t>prevAce</t>
+  </si>
+  <si>
+    <t>nextTab1</t>
+  </si>
+  <si>
+    <t>nextTab2</t>
+  </si>
+  <si>
+    <t>prevTab1</t>
+  </si>
+  <si>
+    <t>prevTab2</t>
+  </si>
+  <si>
+    <t>rns</t>
   </si>
 </sst>
 </file>
@@ -745,4 +782,76 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7D17E4-C3EA-4BBA-A19D-E80A36446237}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>